<commit_message>
Update app to use dedicated tables for colony and nutrition data
Refactor API endpoints and data models to support new, normalized tables for colony metrics, drift events, and threshold labs, replacing direct sheet row access. Update documentation and UI components to reflect these changes.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f1c5c7d3-b1ac-402f-9157-32b255e6b411
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 78819e15-70de-479f-9c73-e7704eb43dc1
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/1f07cee0-0836-4b47-b04f-c5c24638d4fd/f1c5c7d3-b1ac-402f-9157-32b255e6b411/O9L7xSY
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/fixtures/logbook03162026.xlsx
+++ b/fixtures/logbook03162026.xlsx
@@ -514,22 +514,22 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>OAT</v>
+        <v>RIC</v>
       </c>
       <c r="B3" t="str">
-        <v>Oats</v>
+        <v>White Rice</v>
       </c>
       <c r="C3">
-        <v>389</v>
+        <v>130</v>
       </c>
       <c r="D3">
-        <v>17</v>
+        <v>2.7</v>
       </c>
       <c r="E3">
-        <v>66</v>
+        <v>28</v>
       </c>
       <c r="F3">
-        <v>7</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="4">
@@ -546,7 +546,7 @@
         <v>13</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="F4">
         <v>11</v>
@@ -605,8 +605,8 @@
       <c r="D2" t="str">
         <v>CHK</v>
       </c>
-      <c r="E2" t="str">
-        <v>200g</v>
+      <c r="E2">
+        <v>200</v>
       </c>
       <c r="F2">
         <v>330</v>
@@ -618,7 +618,7 @@
         <v>0</v>
       </c>
       <c r="I2">
-        <v>7</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="3">
@@ -632,22 +632,22 @@
         <v>2</v>
       </c>
       <c r="D3" t="str">
-        <v>OAT</v>
-      </c>
-      <c r="E3" t="str">
-        <v>80g</v>
+        <v>RIC</v>
+      </c>
+      <c r="E3">
+        <v>150</v>
       </c>
       <c r="F3">
-        <v>311</v>
+        <v>195</v>
       </c>
       <c r="G3">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H3">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="4">
@@ -663,20 +663,20 @@
       <c r="D4" t="str">
         <v>EGG</v>
       </c>
-      <c r="E4" t="str">
-        <v>3pcs</v>
+      <c r="E4">
+        <v>100</v>
       </c>
       <c r="F4">
-        <v>234</v>
+        <v>155</v>
       </c>
       <c r="G4">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="H4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -718,16 +718,16 @@
         <v>M1</v>
       </c>
       <c r="C2">
-        <v>641</v>
+        <v>525</v>
       </c>
       <c r="D2">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="E2">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="F2">
-        <v>13</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="3">
@@ -738,16 +738,16 @@
         <v>M2</v>
       </c>
       <c r="C3">
-        <v>234</v>
+        <v>155</v>
       </c>
       <c r="D3">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -759,97 +759,151 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>date</v>
       </c>
       <c r="B1" t="str">
-        <v>drift_days</v>
+        <v>phase</v>
       </c>
       <c r="C1" t="str">
-        <v>event</v>
+        <v>drift_type</v>
+      </c>
+      <c r="D1" t="str">
+        <v>drift_source</v>
+      </c>
+      <c r="E1" t="str">
+        <v>confidence</v>
+      </c>
+      <c r="F1" t="str">
+        <v>weighted_drift_score</v>
+      </c>
+      <c r="G1" t="str">
+        <v>watch_flag</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>2026-03-01</v>
       </c>
-      <c r="B2">
-        <v>0</v>
+      <c r="B2" t="str">
+        <v>base</v>
       </c>
       <c r="C2" t="str">
-        <v>FIXTURE-baseline</v>
+        <v>outcome_mismatch</v>
+      </c>
+      <c r="D2" t="str">
+        <v>weight falling during base</v>
+      </c>
+      <c r="E2" t="str">
+        <v>moderate</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2" t="str">
+        <v>watch</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2026-03-10</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
+        <v>2026-03-08</v>
+      </c>
+      <c r="B3" t="str">
+        <v>peak</v>
       </c>
       <c r="C3" t="str">
-        <v>FIXTURE-drift-event</v>
+        <v>schedule_break</v>
+      </c>
+      <c r="D3" t="str">
+        <v>missed training session</v>
+      </c>
+      <c r="E3" t="str">
+        <v>high</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3" t="str">
+        <v>review</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>colony_id</v>
+        <v>metric</v>
       </c>
       <c r="B1" t="str">
-        <v>x</v>
+        <v>value</v>
       </c>
       <c r="C1" t="str">
-        <v>y</v>
+        <v>threshold</v>
       </c>
       <c r="D1" t="str">
-        <v>label</v>
+        <v>status</v>
+      </c>
+      <c r="E1" t="str">
+        <v>recommendation</v>
+      </c>
+      <c r="F1" t="str">
+        <v>confidence</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>C1</v>
-      </c>
-      <c r="B2">
-        <v>0.5</v>
-      </c>
-      <c r="C2">
-        <v>0.3</v>
+        <v>branch_conflict_7d</v>
+      </c>
+      <c r="B2" t="str">
+        <v>4</v>
+      </c>
+      <c r="C2" t="str">
+        <v>&gt;=3</v>
       </c>
       <c r="D2" t="str">
-        <v>FIXTURE-colony-A</v>
+        <v>unstable</v>
+      </c>
+      <c r="E2" t="str">
+        <v>review arbitration weights</v>
+      </c>
+      <c r="F2" t="str">
+        <v>high</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>C2</v>
-      </c>
-      <c r="B3">
-        <v>0.8</v>
-      </c>
-      <c r="C3">
-        <v>0.7</v>
+        <v>sleep_adequacy_proxy</v>
+      </c>
+      <c r="B3" t="str">
+        <v>0.72</v>
+      </c>
+      <c r="C3" t="str">
+        <v>&gt;=0.75</v>
       </c>
       <c r="D3" t="str">
-        <v>FIXTURE-colony-B</v>
+        <v>alert</v>
+      </c>
+      <c r="E3" t="str">
+        <v>increase sleep window</v>
+      </c>
+      <c r="F3" t="str">
+        <v>moderate</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -860,53 +914,53 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>metric</v>
+        <v>threshold_name</v>
       </c>
       <c r="B1" t="str">
-        <v>low</v>
+        <v>current_value</v>
       </c>
       <c r="C1" t="str">
-        <v>mid</v>
+        <v>suggested_value</v>
       </c>
       <c r="D1" t="str">
-        <v>high</v>
+        <v>evidence_count</v>
       </c>
       <c r="E1" t="str">
-        <v>note</v>
+        <v>notes</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>hrv</v>
-      </c>
-      <c r="B2">
-        <v>20</v>
-      </c>
-      <c r="C2">
-        <v>35</v>
+        <v>sleep_adequacy_threshold</v>
+      </c>
+      <c r="B2" t="str">
+        <v>0.75</v>
+      </c>
+      <c r="C2" t="str">
+        <v>0.78</v>
       </c>
       <c r="D2">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="E2" t="str">
-        <v>FIXTURE</v>
+        <v>observe before promotion</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>rhr</v>
-      </c>
-      <c r="B3">
-        <v>45</v>
-      </c>
-      <c r="C3">
-        <v>58</v>
+        <v>hrv_floor</v>
+      </c>
+      <c r="B3" t="str">
+        <v>30</v>
+      </c>
+      <c r="C3" t="str">
+        <v>32</v>
       </c>
       <c r="D3">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="E3" t="str">
-        <v>FIXTURE</v>
+        <v>update after 2 more weeks</v>
       </c>
     </row>
   </sheetData>

</xml_diff>